<commit_message>
Se implementó la sección de cv en vista Acerca del Desarrollador
</commit_message>
<xml_diff>
--- a/reports/ReporteGeneral.xlsx
+++ b/reports/ReporteGeneral.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Nombre</t>
   </si>
@@ -52,6 +52,33 @@
   </si>
   <si>
     <t>5645032022</t>
+  </si>
+  <si>
+    <t>MADELINE</t>
+  </si>
+  <si>
+    <t>madeline_cerezo@hotmail.com</t>
+  </si>
+  <si>
+    <t>5645093031</t>
+  </si>
+  <si>
+    <t>ITAN AARON</t>
+  </si>
+  <si>
+    <t>itan.cerezo@hotmail.com</t>
+  </si>
+  <si>
+    <t>5645041516</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DAVID </t>
+  </si>
+  <si>
+    <t>david_4@hotmail.com</t>
+  </si>
+  <si>
+    <t>5645032932</t>
   </si>
   <si>
     <t>ID Venta</t>
@@ -114,7 +141,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -162,6 +189,39 @@
       </c>
       <c r="C4" t="s" s="0">
         <v>12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -176,19 +236,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>17</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2">
@@ -202,7 +262,7 @@
         <v>4</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Guardando cambios antes de volver al commit bueno
</commit_message>
<xml_diff>
--- a/reports/ReporteGeneral.xlsx
+++ b/reports/ReporteGeneral.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="42">
   <si>
     <t>Nombre</t>
   </si>
@@ -27,58 +27,76 @@
     <t>Celda de prueba</t>
   </si>
   <si>
-    <t>ROGELIO</t>
-  </si>
-  <si>
-    <t>royerch_6@hotmail.com</t>
-  </si>
-  <si>
-    <t>5645031415</t>
-  </si>
-  <si>
-    <t>MARLENE</t>
-  </si>
-  <si>
-    <t>marlene_6@hotmail.com</t>
-  </si>
-  <si>
-    <t>5645032021</t>
-  </si>
-  <si>
-    <t>LAUREN</t>
-  </si>
-  <si>
-    <t>lauren_cerezo@hotmail.com</t>
+    <t>SELENE</t>
+  </si>
+  <si>
+    <t>selene_6@hotmail.com</t>
   </si>
   <si>
     <t>5645032022</t>
   </si>
   <si>
-    <t>MADELINE</t>
-  </si>
-  <si>
-    <t>madeline_cerezo@hotmail.com</t>
-  </si>
-  <si>
-    <t>5645093031</t>
-  </si>
-  <si>
-    <t>ITAN AARON</t>
-  </si>
-  <si>
-    <t>itan.cerezo@hotmail.com</t>
-  </si>
-  <si>
-    <t>5645041516</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAVID </t>
-  </si>
-  <si>
-    <t>david_4@hotmail.com</t>
-  </si>
-  <si>
-    <t>5645032932</t>
+    <t>SEBASTÍAN</t>
+  </si>
+  <si>
+    <t>sebastianbrasil_20@hotmail.com</t>
+  </si>
+  <si>
+    <t>2125032125</t>
+  </si>
+  <si>
+    <t>YOLANDA</t>
+  </si>
+  <si>
+    <t>yolanda_marin56@hotmail.com</t>
+  </si>
+  <si>
+    <t>5554419494</t>
+  </si>
+  <si>
+    <t>ALEJANDRO</t>
+  </si>
+  <si>
+    <t>alejandro_46@hotmail.com</t>
+  </si>
+  <si>
+    <t>5645032130</t>
+  </si>
+  <si>
+    <t>CATARINA</t>
+  </si>
+  <si>
+    <t>catarinacruz@hotmail.com</t>
+  </si>
+  <si>
+    <t>5511090910</t>
+  </si>
+  <si>
+    <t>NATALIA</t>
+  </si>
+  <si>
+    <t>nataliahernandez@hotmail.com</t>
+  </si>
+  <si>
+    <t>5554419495</t>
+  </si>
+  <si>
+    <t>LIAM</t>
+  </si>
+  <si>
+    <t>liamunitedstates@outlook.com</t>
+  </si>
+  <si>
+    <t>2125552123</t>
+  </si>
+  <si>
+    <t>PAMELA</t>
+  </si>
+  <si>
+    <t>pamelaguitierrez@gmail.com</t>
+  </si>
+  <si>
+    <t>5554412025</t>
   </si>
   <si>
     <t>ID Venta</t>
@@ -96,7 +114,31 @@
     <t xml:space="preserve">Celda de prueba </t>
   </si>
   <si>
-    <t>Mon Apr 20 00:00:00 CST 2026</t>
+    <t>Mon Mar 02 09:30:00 CST 2026</t>
+  </si>
+  <si>
+    <t>Thu Apr 02 09:00:00 CST 2026</t>
+  </si>
+  <si>
+    <t>Thu Apr 09 07:00:00 CST 2026</t>
+  </si>
+  <si>
+    <t>Fri Apr 10 09:00:00 CST 2026</t>
+  </si>
+  <si>
+    <t>Sat Apr 11 08:56:00 CST 2026</t>
+  </si>
+  <si>
+    <t>Sun Feb 22 11:00:00 CST 2026</t>
+  </si>
+  <si>
+    <t>Mon Feb 02 17:00:00 CST 2026</t>
+  </si>
+  <si>
+    <t>Thu Jan 01 18:00:00 CST 2026</t>
+  </si>
+  <si>
+    <t>Sat Jan 03 14:30:00 CST 2026</t>
   </si>
 </sst>
 </file>
@@ -141,7 +183,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -222,6 +264,28 @@
       </c>
       <c r="C7" t="s" s="0">
         <v>21</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -231,38 +295,150 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n" s="0">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="B2" t="n" s="0">
-        <v>40000.0</v>
+        <v>12000.0</v>
       </c>
       <c r="C2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B3" t="n" s="0">
+        <v>7000.0</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="B4" t="n" s="0">
+        <v>20000.0</v>
+      </c>
+      <c r="C4" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>27</v>
+      <c r="D4" t="s" s="0">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="B5" t="n" s="0">
+        <v>8500.0</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="B6" t="n" s="0">
+        <v>22000.0</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="B7" t="n" s="0">
+        <v>12000.0</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="B8" t="n" s="0">
+        <v>5400.0</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n" s="0">
+        <v>14.0</v>
+      </c>
+      <c r="B9" t="n" s="0">
+        <v>21340.0</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="B10" t="n" s="0">
+        <v>13030.0</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>